<commit_message>
feat(operation): add operation status batch scheduler
</commit_message>
<xml_diff>
--- a/public/templates/payroll/WeCMS_Payroll_Payment_upload_EN.xlsx
+++ b/public/templates/payroll/WeCMS_Payroll_Payment_upload_EN.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WECMS\Templates\PayrollPayments\NewUpload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\WEBCASH\19. Package\98. 2205 WABOOK\26.06.01 WeCMS\[WeCMS] Service Request\[IMP] Bulk upload templates\Payroll Schedule Payment\20260610\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E4697EC-B069-4359-A5B8-78AF8BAC1953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83FE274B-DC5F-4F2A-9D72-3EB4653F5B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7E411720-582E-4602-B06E-C5399F70CF9D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7E411720-582E-4602-B06E-C5399F70CF9D}"/>
   </bookViews>
   <sheets>
     <sheet name="Payroll" sheetId="1" r:id="rId1"/>
@@ -910,13 +910,13 @@
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1016,7 +1016,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
@@ -1108,6 +1108,18 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1424,17 +1436,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A73773F-D827-4394-BFCF-30EACAF7B583}">
   <dimension ref="A1:I2004"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" zeroHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" zeroHeight="1"/>
   <cols>
-    <col min="1" max="1" width="15.36328125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="29.54296875" style="9" customWidth="1"/>
-    <col min="3" max="3" width="26.1796875" style="9" customWidth="1"/>
-    <col min="4" max="4" width="28.1796875" style="9" customWidth="1"/>
-    <col min="5" max="5" width="22.1796875" style="9" customWidth="1"/>
-    <col min="6" max="6" width="20.1796875" style="9" customWidth="1"/>
-    <col min="7" max="7" width="50.36328125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="29.5703125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" style="26" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="22.140625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" style="9" customWidth="1"/>
+    <col min="7" max="7" width="50.42578125" style="9" customWidth="1"/>
     <col min="8" max="8" width="18" style="9" customWidth="1"/>
-    <col min="9" max="16384" width="8.81640625" style="9"/>
+    <col min="9" max="16384" width="8.85546875" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="2" customFormat="1" ht="21" customHeight="1">
@@ -1468,7 +1480,7 @@
       <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="24" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -1522,7 +1534,7 @@
         <f>IFERROR(INDEX(NOTE!C:C,MATCH(TEXT(A5,"0"),NOTE!B:B,0)),"")</f>
         <v>ShinhanBank</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="25" t="s">
         <v>97</v>
       </c>
       <c r="D5" s="9" t="s">
@@ -13512,7 +13524,7 @@
     <row r="2003" spans="2:2"/>
     <row r="2004" spans="2:2"/>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="wlWV9aS8bEjltDMw9XDdIa4Eeh7CJJz3bLtEBBg4nV1h95JGdb/o3F1SnJ5USx4mfUkOt27PC9Xr/II9315CCQ==" saltValue="Gi6YJIISHkb/sNsoN71xIg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="joux0nfsGDPZFHncjvUAE8DEYQclJAeJVX16MYnEij/XDKOJ2WG5KQf1bhUIMfXiJ06tDBUeWE4alcZ741DzZQ==" saltValue="d38RZcAUlXY2LFzi5o53uA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H2"/>
   </mergeCells>
@@ -13535,14 +13547,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF35AC78-063B-4E06-B357-610DFF13A07B}">
   <dimension ref="B2:E106"/>
-  <sheetFormatPr defaultColWidth="8.08984375" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="2.81640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="8.453125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="19.1796875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="8.08984375" style="2"/>
-    <col min="5" max="5" width="11.90625" style="2" customWidth="1"/>
-    <col min="6" max="16384" width="8.08984375" style="2"/>
+    <col min="1" max="1" width="2.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="8.140625" style="2"/>
+    <col min="5" max="5" width="11.85546875" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="8.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:5">

</xml_diff>